<commit_message>
fix(data): corregir dirección Desquens - # 643 → # 634
</commit_message>
<xml_diff>
--- a/data/referencias/socios/FUENTE_DE_VERDAD_CLUB_738_ENERO_2026.xlsx
+++ b/data/referencias/socios/FUENTE_DE_VERDAD_CLUB_738_ENERO_2026.xlsx
@@ -20138,7 +20138,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>Calle 51-C # 643 x 72 y 72-A</t>
+          <t>Calle 51-C # 634 x 72 y 72-A</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
@@ -20227,7 +20227,7 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>Calle 51-C # 643 x 72 y 72-A</t>
+          <t>Calle 51-C # 634 x 72 y 72-A</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
@@ -20316,7 +20316,7 @@
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>Calle 51-C # 643 x 72 y 72-A</t>
+          <t>Calle 51-C # 634 x 72 y 72-A</t>
         </is>
       </c>
       <c r="J227" t="inlineStr">
@@ -20405,7 +20405,7 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>Calle 51-C # 643 x 72 y 72-A</t>
+          <t>Calle 51-C # 634 x 72 y 72-A</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
@@ -20494,7 +20494,7 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>Calle 51-C # 643 x 72 y 72-A</t>
+          <t>Calle 51-C # 634 x 72 y 72-A</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
@@ -20583,7 +20583,7 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>Calle 51-C # 643 x 72 y 72-A</t>
+          <t>Calle 51-C # 634 x 72 y 72-A</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">

</xml_diff>

<commit_message>
feat(arsenal): alta 3 armas Enrique Gaona + reporte movimientos 2026
- Aprobadas 3 solicitudes de alta para quiquis77@hotmail.com
- Actualizado Excel Fuente de Verdad (filas 299-301)
- Creado docs/MOVIMIENTOS_ARSENAL_2026.md con balance:
  - Altas: 11, Bajas: 1, Movimientos internos: 3, Neto: +10
- Scripts de gestión de arsenal agregados
</commit_message>
<xml_diff>
--- a/data/referencias/socios/FUENTE_DE_VERDAD_CLUB_738_ENERO_2026.xlsx
+++ b/data/referencias/socios/FUENTE_DE_VERDAD_CLUB_738_ENERO_2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S298"/>
+  <dimension ref="A1:S301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18776,11 +18776,6 @@
       <c r="N209" t="n">
         <v>0</v>
       </c>
-      <c r="O209" t="inlineStr"/>
-      <c r="P209" t="inlineStr"/>
-      <c r="Q209" t="inlineStr"/>
-      <c r="R209" t="inlineStr"/>
-      <c r="S209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -19116,7 +19111,6 @@
           <t>BERETTA</t>
         </is>
       </c>
-      <c r="Q213" t="inlineStr"/>
       <c r="R213" t="n">
         <v>92070</v>
       </c>
@@ -21315,11 +21309,6 @@
       <c r="N238" t="n">
         <v>0</v>
       </c>
-      <c r="O238" t="inlineStr"/>
-      <c r="P238" t="inlineStr"/>
-      <c r="Q238" t="inlineStr"/>
-      <c r="R238" t="inlineStr"/>
-      <c r="S238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -21556,11 +21545,6 @@
       <c r="N241" t="n">
         <v>0</v>
       </c>
-      <c r="O241" t="inlineStr"/>
-      <c r="P241" t="inlineStr"/>
-      <c r="Q241" t="inlineStr"/>
-      <c r="R241" t="inlineStr"/>
-      <c r="S241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -21888,11 +21872,6 @@
       <c r="N245" t="n">
         <v>0</v>
       </c>
-      <c r="O245" t="inlineStr"/>
-      <c r="P245" t="inlineStr"/>
-      <c r="Q245" t="inlineStr"/>
-      <c r="R245" t="inlineStr"/>
-      <c r="S245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -23460,11 +23439,6 @@
       <c r="N263" t="n">
         <v>0</v>
       </c>
-      <c r="O263" t="inlineStr"/>
-      <c r="P263" t="inlineStr"/>
-      <c r="Q263" t="inlineStr"/>
-      <c r="R263" t="inlineStr"/>
-      <c r="S263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -24680,11 +24654,6 @@
       <c r="N277" t="n">
         <v>0</v>
       </c>
-      <c r="O277" t="inlineStr"/>
-      <c r="P277" t="inlineStr"/>
-      <c r="Q277" t="inlineStr"/>
-      <c r="R277" t="inlineStr"/>
-      <c r="S277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -24747,11 +24716,6 @@
       <c r="N278" t="n">
         <v>0</v>
       </c>
-      <c r="O278" t="inlineStr"/>
-      <c r="P278" t="inlineStr"/>
-      <c r="Q278" t="inlineStr"/>
-      <c r="R278" t="inlineStr"/>
-      <c r="S278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -24901,11 +24865,6 @@
       <c r="N280" t="n">
         <v>0</v>
       </c>
-      <c r="O280" t="inlineStr"/>
-      <c r="P280" t="inlineStr"/>
-      <c r="Q280" t="inlineStr"/>
-      <c r="R280" t="inlineStr"/>
-      <c r="S280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -24968,15 +24927,8 @@
       <c r="N281" t="n">
         <v>0</v>
       </c>
-      <c r="O281" t="inlineStr"/>
-      <c r="P281" t="inlineStr"/>
-      <c r="Q281" t="inlineStr"/>
-      <c r="R281" t="inlineStr"/>
-      <c r="S281" t="inlineStr"/>
     </row>
     <row r="282">
-      <c r="A282" t="inlineStr"/>
-      <c r="B282" t="inlineStr"/>
       <c r="C282" t="n">
         <v>199</v>
       </c>
@@ -24990,7 +24942,6 @@
           <t>jrgardoni@gmail.com</t>
         </is>
       </c>
-      <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
           <t>jrgardoni@gmail.com</t>
@@ -25001,11 +24952,6 @@
           <t>2021-12-14</t>
         </is>
       </c>
-      <c r="I282" t="inlineStr"/>
-      <c r="J282" t="inlineStr"/>
-      <c r="K282" t="inlineStr"/>
-      <c r="L282" t="inlineStr"/>
-      <c r="M282" t="inlineStr"/>
       <c r="N282" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25038,8 +24984,6 @@
       </c>
     </row>
     <row r="283">
-      <c r="A283" t="inlineStr"/>
-      <c r="B283" t="inlineStr"/>
       <c r="C283" t="n">
         <v>199</v>
       </c>
@@ -25053,7 +24997,6 @@
           <t>jrgardoni@gmail.com</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>jrgardoni@gmail.com</t>
@@ -25064,11 +25007,6 @@
           <t>2021-12-14</t>
         </is>
       </c>
-      <c r="I283" t="inlineStr"/>
-      <c r="J283" t="inlineStr"/>
-      <c r="K283" t="inlineStr"/>
-      <c r="L283" t="inlineStr"/>
-      <c r="M283" t="inlineStr"/>
       <c r="N283" t="inlineStr">
         <is>
           <t>RIFLE</t>
@@ -25101,8 +25039,6 @@
       </c>
     </row>
     <row r="284">
-      <c r="A284" t="inlineStr"/>
-      <c r="B284" t="inlineStr"/>
       <c r="C284" t="n">
         <v>199</v>
       </c>
@@ -25116,7 +25052,6 @@
           <t>jrgardoni@gmail.com</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
           <t>jrgardoni@gmail.com</t>
@@ -25127,11 +25062,6 @@
           <t>2021-12-14</t>
         </is>
       </c>
-      <c r="I284" t="inlineStr"/>
-      <c r="J284" t="inlineStr"/>
-      <c r="K284" t="inlineStr"/>
-      <c r="L284" t="inlineStr"/>
-      <c r="M284" t="inlineStr"/>
       <c r="N284" t="inlineStr">
         <is>
           <t>RIFLE</t>
@@ -25164,8 +25094,6 @@
       </c>
     </row>
     <row r="285">
-      <c r="A285" t="inlineStr"/>
-      <c r="B285" t="inlineStr"/>
       <c r="C285" t="n">
         <v>199</v>
       </c>
@@ -25179,7 +25107,6 @@
           <t>jrgardoni@gmail.com</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
           <t>jrgardoni@gmail.com</t>
@@ -25190,11 +25117,6 @@
           <t>2021-12-14</t>
         </is>
       </c>
-      <c r="I285" t="inlineStr"/>
-      <c r="J285" t="inlineStr"/>
-      <c r="K285" t="inlineStr"/>
-      <c r="L285" t="inlineStr"/>
-      <c r="M285" t="inlineStr"/>
       <c r="N285" t="inlineStr">
         <is>
           <t>RIFLE</t>
@@ -25227,8 +25149,6 @@
       </c>
     </row>
     <row r="286">
-      <c r="A286" t="inlineStr"/>
-      <c r="B286" t="inlineStr"/>
       <c r="C286" t="n">
         <v>199</v>
       </c>
@@ -25242,7 +25162,6 @@
           <t>jrgardoni@gmail.com</t>
         </is>
       </c>
-      <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
           <t>jrgardoni@gmail.com</t>
@@ -25253,11 +25172,6 @@
           <t>2021-12-14</t>
         </is>
       </c>
-      <c r="I286" t="inlineStr"/>
-      <c r="J286" t="inlineStr"/>
-      <c r="K286" t="inlineStr"/>
-      <c r="L286" t="inlineStr"/>
-      <c r="M286" t="inlineStr"/>
       <c r="N286" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25290,8 +25204,6 @@
       </c>
     </row>
     <row r="287">
-      <c r="A287" t="inlineStr"/>
-      <c r="B287" t="inlineStr"/>
       <c r="C287" t="n">
         <v>199</v>
       </c>
@@ -25305,7 +25217,6 @@
           <t>jrgardoni@gmail.com</t>
         </is>
       </c>
-      <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
           <t>jrgardoni@gmail.com</t>
@@ -25316,11 +25227,6 @@
           <t>2021-12-14</t>
         </is>
       </c>
-      <c r="I287" t="inlineStr"/>
-      <c r="J287" t="inlineStr"/>
-      <c r="K287" t="inlineStr"/>
-      <c r="L287" t="inlineStr"/>
-      <c r="M287" t="inlineStr"/>
       <c r="N287" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25353,8 +25259,6 @@
       </c>
     </row>
     <row r="288">
-      <c r="A288" t="inlineStr"/>
-      <c r="B288" t="inlineStr"/>
       <c r="C288" t="n">
         <v>199</v>
       </c>
@@ -25368,7 +25272,6 @@
           <t>jrgardoni@gmail.com</t>
         </is>
       </c>
-      <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
           <t>jrgardoni@gmail.com</t>
@@ -25379,11 +25282,6 @@
           <t>2021-12-14</t>
         </is>
       </c>
-      <c r="I288" t="inlineStr"/>
-      <c r="J288" t="inlineStr"/>
-      <c r="K288" t="inlineStr"/>
-      <c r="L288" t="inlineStr"/>
-      <c r="M288" t="inlineStr"/>
       <c r="N288" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25416,8 +25314,6 @@
       </c>
     </row>
     <row r="289">
-      <c r="A289" t="inlineStr"/>
-      <c r="B289" t="inlineStr"/>
       <c r="C289" t="n">
         <v>212</v>
       </c>
@@ -25431,7 +25327,6 @@
           <t>arechiga@jogarplastics.com</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
           <t>arechiga@jogarplastics.com</t>
@@ -25442,11 +25337,6 @@
           <t>2024-06-28</t>
         </is>
       </c>
-      <c r="I289" t="inlineStr"/>
-      <c r="J289" t="inlineStr"/>
-      <c r="K289" t="inlineStr"/>
-      <c r="L289" t="inlineStr"/>
-      <c r="M289" t="inlineStr"/>
       <c r="N289" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25479,8 +25369,6 @@
       </c>
     </row>
     <row r="290">
-      <c r="A290" t="inlineStr"/>
-      <c r="B290" t="inlineStr"/>
       <c r="C290" t="n">
         <v>212</v>
       </c>
@@ -25494,7 +25382,6 @@
           <t>arechiga@jogarplastics.com</t>
         </is>
       </c>
-      <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
           <t>arechiga@jogarplastics.com</t>
@@ -25505,11 +25392,6 @@
           <t>2024-06-28</t>
         </is>
       </c>
-      <c r="I290" t="inlineStr"/>
-      <c r="J290" t="inlineStr"/>
-      <c r="K290" t="inlineStr"/>
-      <c r="L290" t="inlineStr"/>
-      <c r="M290" t="inlineStr"/>
       <c r="N290" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25542,8 +25424,6 @@
       </c>
     </row>
     <row r="291">
-      <c r="A291" t="inlineStr"/>
-      <c r="B291" t="inlineStr"/>
       <c r="C291" t="n">
         <v>212</v>
       </c>
@@ -25557,7 +25437,6 @@
           <t>arechiga@jogarplastics.com</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
           <t>arechiga@jogarplastics.com</t>
@@ -25568,11 +25447,6 @@
           <t>2024-06-28</t>
         </is>
       </c>
-      <c r="I291" t="inlineStr"/>
-      <c r="J291" t="inlineStr"/>
-      <c r="K291" t="inlineStr"/>
-      <c r="L291" t="inlineStr"/>
-      <c r="M291" t="inlineStr"/>
       <c r="N291" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25605,8 +25479,6 @@
       </c>
     </row>
     <row r="292">
-      <c r="A292" t="inlineStr"/>
-      <c r="B292" t="inlineStr"/>
       <c r="C292" t="n">
         <v>183</v>
       </c>
@@ -25615,8 +25487,6 @@
           <t>CELESTINO SANCHEZ FERNANDEZ</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr"/>
-      <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
           <t>tinosanchezf@yahoo.com.mx</t>
@@ -25627,11 +25497,6 @@
           <t>2020-02-24</t>
         </is>
       </c>
-      <c r="I292" t="inlineStr"/>
-      <c r="J292" t="inlineStr"/>
-      <c r="K292" t="inlineStr"/>
-      <c r="L292" t="inlineStr"/>
-      <c r="M292" t="inlineStr"/>
       <c r="N292" t="inlineStr">
         <is>
           <t>RIFLE</t>
@@ -25662,8 +25527,6 @@
       </c>
     </row>
     <row r="293">
-      <c r="A293" t="inlineStr"/>
-      <c r="B293" t="inlineStr"/>
       <c r="C293" t="n">
         <v>183</v>
       </c>
@@ -25672,8 +25535,6 @@
           <t>CELESTINO SANCHEZ FERNANDEZ</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr"/>
-      <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
           <t>tinosanchezf@yahoo.com.mx</t>
@@ -25684,11 +25545,6 @@
           <t>2020-02-24</t>
         </is>
       </c>
-      <c r="I293" t="inlineStr"/>
-      <c r="J293" t="inlineStr"/>
-      <c r="K293" t="inlineStr"/>
-      <c r="L293" t="inlineStr"/>
-      <c r="M293" t="inlineStr"/>
       <c r="N293" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25721,8 +25577,6 @@
       </c>
     </row>
     <row r="294">
-      <c r="A294" t="inlineStr"/>
-      <c r="B294" t="inlineStr"/>
       <c r="C294" t="n">
         <v>183</v>
       </c>
@@ -25731,8 +25585,6 @@
           <t>CELESTINO SANCHEZ FERNANDEZ</t>
         </is>
       </c>
-      <c r="E294" t="inlineStr"/>
-      <c r="F294" t="inlineStr"/>
       <c r="G294" t="inlineStr">
         <is>
           <t>tinosanchezf@yahoo.com.mx</t>
@@ -25743,11 +25595,6 @@
           <t>2020-02-24</t>
         </is>
       </c>
-      <c r="I294" t="inlineStr"/>
-      <c r="J294" t="inlineStr"/>
-      <c r="K294" t="inlineStr"/>
-      <c r="L294" t="inlineStr"/>
-      <c r="M294" t="inlineStr"/>
       <c r="N294" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25780,8 +25627,6 @@
       </c>
     </row>
     <row r="295">
-      <c r="A295" t="inlineStr"/>
-      <c r="B295" t="inlineStr"/>
       <c r="C295" t="n">
         <v>183</v>
       </c>
@@ -25790,8 +25635,6 @@
           <t>CELESTINO SANCHEZ FERNANDEZ</t>
         </is>
       </c>
-      <c r="E295" t="inlineStr"/>
-      <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
           <t>tinosanchezf@yahoo.com.mx</t>
@@ -25802,11 +25645,6 @@
           <t>2020-02-24</t>
         </is>
       </c>
-      <c r="I295" t="inlineStr"/>
-      <c r="J295" t="inlineStr"/>
-      <c r="K295" t="inlineStr"/>
-      <c r="L295" t="inlineStr"/>
-      <c r="M295" t="inlineStr"/>
       <c r="N295" t="inlineStr">
         <is>
           <t>PISTOLA</t>
@@ -25839,7 +25677,6 @@
       </c>
     </row>
     <row r="296">
-      <c r="A296" t="inlineStr"/>
       <c r="B296" t="inlineStr">
         <is>
           <t>Calle 32 x 9 Cedro, Tablaje 23222, Loc. Tixcuytun, Mérida, YUCATÁN CP97305</t>
@@ -25869,19 +25706,9 @@
       <c r="H296" t="n">
         <v>25568.75053275463</v>
       </c>
-      <c r="I296" t="inlineStr"/>
-      <c r="J296" t="inlineStr"/>
-      <c r="K296" t="inlineStr"/>
-      <c r="L296" t="inlineStr"/>
-      <c r="M296" t="inlineStr"/>
       <c r="N296" t="n">
         <v>0</v>
       </c>
-      <c r="O296" t="inlineStr"/>
-      <c r="P296" t="inlineStr"/>
-      <c r="Q296" t="inlineStr"/>
-      <c r="R296" t="inlineStr"/>
-      <c r="S296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -26058,6 +25885,273 @@
       <c r="S298" t="inlineStr">
         <is>
           <t>A3903742</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>738</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>CALLE 50 No. 531-E x 69 y 71, CENTRO, 97000 MÉRIDA, YUC.</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>195</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>ENRIQUE GAONA CASTAÑEDA</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>GACE770131HDFNFN04</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>5520985073</v>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>quiquis77@hotmail.com</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>2022-03-03</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>C. 137 No. 1295</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>FRACC. DIAMANTE OPICHEN</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>MÉRIDA</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>YUCATÁN</t>
+        </is>
+      </c>
+      <c r="M299" t="n">
+        <v>97249</v>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>RIFLE</t>
+        </is>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>.22 LR</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>CESKA ZBROJOVKA</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>CZ 512</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>J100907</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>A3900899</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>738</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>CALLE 50 No. 531-E x 69 y 71, CENTRO, 97000 MÉRIDA, YUC.</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>195</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>ENRIQUE GAONA CASTAÑEDA</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>GACE770131HDFNFN04</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>5520985073</v>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>quiquis77@hotmail.com</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>2022-03-03</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>C. 137 No. 1295</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>FRACC. DIAMANTE OPICHEN</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>MÉRIDA</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>YUCATÁN</t>
+        </is>
+      </c>
+      <c r="M300" t="n">
+        <v>97249</v>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>PISTOLA</t>
+        </is>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>.380</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>BERETTA</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>80 X</t>
+        </is>
+      </c>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>Y014871X</t>
+        </is>
+      </c>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>A3900898</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>738</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>CALLE 50 No. 531-E x 69 y 71, CENTRO, 97000 MÉRIDA, YUC.</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>195</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>ENRIQUE GAONA CASTAÑEDA</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>GACE770131HDFNFN04</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>5520985073</v>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>quiquis77@hotmail.com</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>2022-03-03</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>C. 137 No. 1295</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>FRACC. DIAMANTE OPICHEN</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>MÉRIDA</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>YUCATÁN</t>
+        </is>
+      </c>
+      <c r="M301" t="n">
+        <v>97249</v>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>PISTOLA</t>
+        </is>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>.22 LR</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>SIG SAUER</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>P322</t>
+        </is>
+      </c>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>73A192310</t>
+        </is>
+      </c>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>A3916770</t>
         </is>
       </c>
     </row>

</xml_diff>